<commit_message>
Updated Excel Data Again.
</commit_message>
<xml_diff>
--- a/12627062.xlsx
+++ b/12627062.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e613dd4f33c0853c/Documents/Computer Application/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{732F1569-5717-4D99-B03F-E6BC4F58C405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54D0C80A-AF27-436C-BA7B-C6B860FBF886}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{732F1569-5717-4D99-B03F-E6BC4F58C405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88CCC49A-8995-4F14-A185-439B21126C7B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="99">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -626,6 +626,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3101,26 +3105,50 @@
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+      <c r="A49" s="8">
+        <v>46294</v>
+      </c>
+      <c r="B49" s="14">
+        <v>60</v>
+      </c>
+      <c r="C49" s="14">
+        <v>30</v>
+      </c>
+      <c r="D49" s="14">
+        <v>120</v>
+      </c>
+      <c r="E49" s="14">
+        <v>220</v>
+      </c>
+      <c r="F49" s="14">
+        <v>0</v>
+      </c>
+      <c r="G49" s="14">
+        <v>0</v>
+      </c>
+      <c r="H49" s="14">
+        <v>220</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>650</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
+        <v>790</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="13"/>
@@ -10875,12 +10903,12 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J47 J49:J401">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
+  <conditionalFormatting sqref="J6:J48 J50:J401">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J48">
+  <conditionalFormatting sqref="J49">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
update my excel sheet.
</commit_message>
<xml_diff>
--- a/12627062.xlsx
+++ b/12627062.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e613dd4f33c0853c/Documents/Computer Application/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{732F1569-5717-4D99-B03F-E6BC4F58C405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD2CD083-D0B1-435C-A978-D494B5D6757B}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{732F1569-5717-4D99-B03F-E6BC4F58C405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44A101A8-FEEB-441B-9FC9-BFB6140931BA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="101">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -337,6 +337,9 @@
   </si>
   <si>
     <t>Not a good day.</t>
+  </si>
+  <si>
+    <t>feeling low.</t>
   </si>
 </sst>
 </file>
@@ -3188,26 +3191,50 @@
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+      <c r="A51" s="8">
+        <v>46296</v>
+      </c>
+      <c r="B51" s="14">
+        <v>380</v>
+      </c>
+      <c r="C51" s="14">
+        <v>60</v>
+      </c>
+      <c r="D51" s="14">
+        <v>260</v>
+      </c>
+      <c r="E51" s="14">
+        <v>180</v>
+      </c>
+      <c r="F51" s="14">
+        <v>0</v>
+      </c>
+      <c r="G51" s="14">
+        <v>0</v>
+      </c>
+      <c r="H51" s="14">
+        <v>180</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>1060</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
+        <v>380</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N51" s="17" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>

</xml_diff>

<commit_message>
update Excel sheet data.
</commit_message>
<xml_diff>
--- a/12627062.xlsx
+++ b/12627062.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e613dd4f33c0853c/Documents/Computer Application/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{732F1569-5717-4D99-B03F-E6BC4F58C405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D22826C6-BF4F-4F46-916F-3CA189127FC5}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{732F1569-5717-4D99-B03F-E6BC4F58C405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28DA3548-7F03-4D14-ACAC-B0D1DC0220D7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="103">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -343,6 +343,9 @@
   </si>
   <si>
     <t>fruitful day.</t>
+  </si>
+  <si>
+    <t>stressed day.</t>
   </si>
 </sst>
 </file>
@@ -3332,26 +3335,50 @@
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+      <c r="A54" s="8">
+        <v>46299</v>
+      </c>
+      <c r="B54" s="14">
+        <v>380</v>
+      </c>
+      <c r="C54" s="14">
+        <v>45</v>
+      </c>
+      <c r="D54" s="14">
+        <v>240</v>
+      </c>
+      <c r="E54" s="14">
+        <v>180</v>
+      </c>
+      <c r="F54" s="14">
+        <v>0</v>
+      </c>
+      <c r="G54" s="14">
+        <v>0</v>
+      </c>
+      <c r="H54" s="14">
+        <v>120</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>965</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="17"/>
+        <v>475</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M54" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N54" s="17" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="13"/>

</xml_diff>